<commit_message>
Fix: OpenAI API key explicit passing, add README, deployment ready
</commit_message>
<xml_diff>
--- a/Reports/ChurnReport_2026-05-14.xlsx
+++ b/Reports/ChurnReport_2026-05-14.xlsx
@@ -75,7 +75,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -107,6 +107,11 @@
         <fgColor rgb="00FFB3B3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -134,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -159,6 +164,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -546,7 +554,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 14-May-2026 13:12  |  Records: 10  |  Currency: INR (₹)</t>
+          <t>Generated: 14-May-2026 14:01  |  Records: 100  |  Currency: INR (₹)</t>
         </is>
       </c>
     </row>
@@ -577,7 +585,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Average NPS Score</t>
+          <t>Churn Risk Customers</t>
         </is>
       </c>
     </row>
@@ -589,7 +597,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>23</t>
         </is>
       </c>
     </row>
@@ -601,7 +609,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>WARNING</t>
         </is>
       </c>
     </row>
@@ -613,7 +621,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>{'average_balance': '₹12,561,290.21', 'average_credit_score': '668.7'}</t>
+          <t>{'Average NPS Score': '5.67', 'High Risk Customers with NPS &lt;= 3': '23', 'Anomalies Detected': '24'}</t>
         </is>
       </c>
     </row>
@@ -627,7 +635,7 @@
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1. Finding 1 — All churned customers are from the Premium segment and are located in Delhi.</t>
+          <t>1. Finding 1 — Out of 100 sampled customers, 23 are at high churn risk, exceeding the NPS risk floor.</t>
         </is>
       </c>
       <c r="B12" s="6" t="n"/>
@@ -635,7 +643,7 @@
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>2. Finding 2 — Average NPS score is critically low at 1.7, with 90% at or below the risk floor.</t>
+          <t>2. Finding 2 — A significant number of high-risk customers belong to the Basic segment with credit scores below 500.</t>
         </is>
       </c>
       <c r="B13" s="5" t="n"/>
@@ -643,7 +651,7 @@
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>3. Finding 3 — Despite high balances, the average tenure is only 2.9 years, indicating potential dissatisfaction early in the customer lifecycle.</t>
+          <t>3. Finding 3 — There is a notable presence of transaction anomalies, affecting 24% of the sampled customers.</t>
         </is>
       </c>
       <c r="B14" s="6" t="n"/>
@@ -668,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -677,14 +685,6 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -695,628 +695,2244 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>nps_score</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>credit_score</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>gender</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>age</t>
-        </is>
-      </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>tenure</t>
+          <t>emi_status</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>balance</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>products_number</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>estimated_salary</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>nps_score</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>segment</t>
-        </is>
-      </c>
-      <c r="L1" s="4" t="inlineStr">
-        <is>
-          <t>joining_date</t>
-        </is>
-      </c>
-      <c r="M1" s="4" t="inlineStr">
-        <is>
-          <t>account_type</t>
-        </is>
-      </c>
-      <c r="N1" s="4" t="inlineStr">
-        <is>
-          <t>kyc_status</t>
+          <t>is_anomaly</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>15794171</v>
+        <v>15634602</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>475</v>
+        <v>0</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>0</v>
+        <v>619</v>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>12658413.69</v>
-      </c>
-      <c r="G2" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="H2" s="5" t="n">
-        <v>2623151.5</v>
-      </c>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>24-10-2025</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="n">
-        <v>15703793</v>
+        <v>15701354</v>
       </c>
       <c r="B3" s="6" t="n">
-        <v>738</v>
+        <v>2</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>58</v>
+        <v>699</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>2</v>
+        <v/>
       </c>
       <c r="F3" s="6" t="n">
-        <v>12609520.08</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>2675087.52</v>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" s="6" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>13-03-2024</t>
-        </is>
-      </c>
-      <c r="M3" s="6" t="inlineStr">
-        <is>
-          <t>Salary</t>
-        </is>
-      </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>15637753</v>
+        <v>15737173</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>751</v>
+        <v>7</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>50</v>
+        <v>497</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>2</v>
+        <v/>
       </c>
       <c r="F4" s="5" t="n">
-        <v>9134637.41</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>7279005.25</v>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>10-08-2023</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>Salary</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
-        <v>15694408</v>
+        <v>15737173</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>749</v>
+        <v>7</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>40</v>
+        <v>497</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="F5" s="6" t="n">
-        <v>13132299.85</v>
-      </c>
-      <c r="G5" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>17239609</v>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>22-11-2024</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>15745844</v>
+        <v>15737173</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>642</v>
+        <v>7</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>40</v>
+        <v>497</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>6</v>
+        <v/>
       </c>
       <c r="F6" s="5" t="n">
-        <v>12209494.76</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>8117435.4</v>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>10-11-2019</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>Salary</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>15674551</v>
+        <v>15737173</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>535</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>40</v>
+        <v>497</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>7</v>
+        <v/>
       </c>
       <c r="F7" s="6" t="n">
-        <v>10536402.82</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>766338.01</v>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L7" s="6" t="inlineStr">
-        <is>
-          <t>15-05-2018</t>
-        </is>
-      </c>
-      <c r="M7" s="6" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>15593782</v>
+        <v>15737173</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>816</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>38</v>
+        <v>497</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>5</v>
+        <v/>
       </c>
       <c r="F8" s="5" t="n">
-        <v>12339248.55</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>6779276</v>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>12-06-2020</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>15683625</v>
+        <v>15737173</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>703</v>
+        <v>7</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>37</v>
+        <v>497</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>1</v>
+        <v/>
       </c>
       <c r="F9" s="6" t="n">
-        <v>14119568.9</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>1944939.83</v>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
-        <is>
-          <t>08-06-2024</t>
-        </is>
-      </c>
-      <c r="M9" s="6" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>15585865</v>
+        <v>15737173</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>673</v>
+        <v>7</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>38</v>
+        <v>497</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>2</v>
+        <v/>
       </c>
       <c r="F10" s="5" t="n">
-        <v>16033437.82</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>12718498.34</v>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>Premium</t>
-        </is>
-      </c>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>05-08-2023</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>Savings</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>15682048</v>
+        <v>15737173</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>605</v>
+        <v>7</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Basic</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>51</v>
+        <v>497</v>
       </c>
       <c r="E11" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>497</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>497</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>497</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>497</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>15737173</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B37" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E38" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="n">
+        <v>476</v>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>15632264</v>
+      </c>
+      <c r="B41" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>476</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n">
+        <v>15600882</v>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n">
+        <v>635</v>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>15737452</v>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>653</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n">
+        <v>15788218</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="n">
+        <v>549</v>
+      </c>
+      <c r="E44" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F44" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>15568982</v>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>726</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
+        <v>15568982</v>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="n">
+        <v>726</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F46" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>15738191</v>
+      </c>
+      <c r="B47" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>12839878.18</v>
-      </c>
-      <c r="G11" s="6" t="n">
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>577</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F47" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="6" t="n">
-        <v>6327186.43</v>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>Delhi</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="n">
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n">
+        <v>15736816</v>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="n">
+        <v>756</v>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>15732963</v>
+      </c>
+      <c r="B49" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>722</v>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E50" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B51" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E52" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F52" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B53" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E54" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B55" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E56" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B57" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B59" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E60" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F60" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B61" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E62" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F62" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B63" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F64" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B65" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E66" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F66" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B67" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B68" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="n">
+        <v>472</v>
+      </c>
+      <c r="E68" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F68" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>15619360</v>
+      </c>
+      <c r="B69" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>472</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n">
+        <v>15738148</v>
+      </c>
+      <c r="B70" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>465</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F70" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n">
+        <v>15602280</v>
+      </c>
+      <c r="B71" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>829</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n">
+        <v>15647091</v>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="n">
+        <v>725</v>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F72" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n">
+        <v>15773469</v>
+      </c>
+      <c r="B73" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>687</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n">
+        <v>15703793</v>
+      </c>
+      <c r="B74" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="C74" s="5" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr">
-        <is>
-          <t>29-10-2022</t>
-        </is>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
+      <c r="D74" s="5" t="n">
+        <v>738</v>
+      </c>
+      <c r="E74" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F74" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>15812518</v>
+      </c>
+      <c r="B75" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>657</v>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n">
+        <v>15614049</v>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="n">
+        <v>664</v>
+      </c>
+      <c r="E76" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F76" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>15575185</v>
+      </c>
+      <c r="B77" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>757</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B78" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E78" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F78" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B79" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E80" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F80" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B81" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B82" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E82" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F82" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E84" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F84" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B85" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E86" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F86" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B87" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E88" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F88" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B89" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B90" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E90" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F90" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B91" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>493</v>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n">
+        <v>15738751</v>
+      </c>
+      <c r="B92" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="n">
+        <v>493</v>
+      </c>
+      <c r="E92" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F92" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n">
+        <v>15625759</v>
+      </c>
+      <c r="B93" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>729</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n">
+        <v>15625759</v>
+      </c>
+      <c r="B94" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="E94" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F94" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n">
+        <v>15622897</v>
+      </c>
+      <c r="B95" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>646</v>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n">
+        <v>15809248</v>
+      </c>
+      <c r="B96" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="n">
+        <v>524</v>
+      </c>
+      <c r="E96" s="5" t="n">
+        <v/>
+      </c>
+      <c r="F96" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n">
+        <v>15738721</v>
+      </c>
+      <c r="B97" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C97" s="6" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>773</v>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v/>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n">
+        <v>15633059</v>
+      </c>
+      <c r="B98" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D98" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="E98" s="5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n">
+        <v>15633059</v>
+      </c>
+      <c r="B99" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>413</v>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n">
+        <v>15633059</v>
+      </c>
+      <c r="B100" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D100" s="5" t="n">
+        <v>413</v>
+      </c>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n">
+        <v>15633059</v>
+      </c>
+      <c r="B101" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Basic</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>413</v>
+      </c>
+      <c r="E101" s="6" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1354,7 +2970,7 @@
     <row r="4" ht="50" customHeight="1">
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>In the Premium segment from Delhi, a group of high-value customers with low NPS scores is exhibiting churn, suggesting dissatisfaction possibly related to service or experience. This group has a notably low tenure and high average balance, making it crucial to address their concerns to prevent future losses.</t>
+          <t>The analysis identifies a significant churn risk primarily attributed to customers with low NPS scores and missed EMI payments. The overall churn risk remains a WARNING as it borders the critical threshold due to high-risk customers in the Basic segment.</t>
         </is>
       </c>
     </row>
@@ -1368,8 +2984,8 @@
     <row r="7" ht="50" customHeight="1">
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>1. Initiate targeted retention initiatives including personalized engagement for Premium segment customers in Delhi.
-2. Conduct detailed surveys or interviews with churned customers to identify primary dissatisfaction drivers and address them urgently.</t>
+          <t>1. Target high-risk customers with tailored strategies to improve their NPS and corresponding loyalty.
+2. Implement risk mitigation strategies for the Basic segment customers with low credit scores and frequent missed EMI payments.</t>
         </is>
       </c>
     </row>
@@ -1450,7 +3066,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>9 customer(s) at or below NPS risk floor (3/10) — churn risk elevated</t>
+          <t>2 customer(s) with extreme dissatisfaction (NPS 0 or 1 out of 10) — highest churn probability</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -1465,34 +3081,34 @@
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>Cross-reference with EMI data and initiate retention outreach.</t>
+          <t>Immediate personal outreach. Assign to senior relationship manager.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>ANO-002</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>5 customer(s) with extreme dissatisfaction (NPS 0 or 1 out of 10) — highest churn probability</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>Immediate personal outreach. Assign to senior relationship manager.</t>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>77 customers in high-risk zone: Basic segment AND credit_score &lt; 500. Churned: N/A</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Review credit risk exposure. Consider proactive outreach.</t>
         </is>
       </c>
     </row>
@@ -1565,7 +3181,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -1637,7 +3253,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>14-May-2026 13:12</t>
+          <t>14-May-2026 14:01</t>
         </is>
       </c>
     </row>
@@ -1654,7 +3270,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>CONFIDENTIAL — BankSight AI Internal Report</t>
         </is>

</xml_diff>